<commit_message>
Add VSCode terminal profile for MSVC Command Prompt
- Created a new settings.json file in the .vscode directory.
- Configured a terminal profile for Command Prompt (MSVC) to initialize the Visual Studio environment.
- Set the default terminal profile to the newly created Command Prompt (MSVC).
</commit_message>
<xml_diff>
--- a/T01_bo_prototype/data/experiments.xlsx
+++ b/T01_bo_prototype/data/experiments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,6 +963,336 @@
         <v>176.411867046571</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1754</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1491</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1813</v>
+      </c>
+      <c r="E12" t="n">
+        <v>47</v>
+      </c>
+      <c r="F12" t="n">
+        <v>70</v>
+      </c>
+      <c r="G12" t="n">
+        <v>81</v>
+      </c>
+      <c r="H12" t="n">
+        <v>27</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1415</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1636</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1796</v>
+      </c>
+      <c r="E13" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" t="n">
+        <v>56</v>
+      </c>
+      <c r="G13" t="n">
+        <v>88</v>
+      </c>
+      <c r="H13" t="n">
+        <v>27</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1439</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1478</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1514</v>
+      </c>
+      <c r="E14" t="n">
+        <v>77</v>
+      </c>
+      <c r="F14" t="n">
+        <v>41</v>
+      </c>
+      <c r="G14" t="n">
+        <v>77</v>
+      </c>
+      <c r="H14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1463</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>75</v>
+      </c>
+      <c r="F15" t="n">
+        <v>96</v>
+      </c>
+      <c r="G15" t="n">
+        <v>78</v>
+      </c>
+      <c r="H15" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1434</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>100</v>
+      </c>
+      <c r="F16" t="n">
+        <v>40</v>
+      </c>
+      <c r="G16" t="n">
+        <v>88</v>
+      </c>
+      <c r="H16" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>100</v>
+      </c>
+      <c r="F17" t="n">
+        <v>40</v>
+      </c>
+      <c r="G17" t="n">
+        <v>87</v>
+      </c>
+      <c r="H17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1473</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" t="n">
+        <v>72</v>
+      </c>
+      <c r="G18" t="n">
+        <v>82</v>
+      </c>
+      <c r="H18" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1454</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1412</v>
+      </c>
+      <c r="E19" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G19" t="n">
+        <v>78</v>
+      </c>
+      <c r="H19" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1702</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E20" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" t="n">
+        <v>100</v>
+      </c>
+      <c r="G20" t="n">
+        <v>94</v>
+      </c>
+      <c r="H20" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1441</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1708</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E21" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" t="n">
+        <v>44</v>
+      </c>
+      <c r="G21" t="n">
+        <v>89</v>
+      </c>
+      <c r="H21" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>